<commit_message>
Created new scripts and updated existing scripts
</commit_message>
<xml_diff>
--- a/testExecution/api-e2e-testing/API-TestData/728300_Organization.xlsx
+++ b/testExecution/api-e2e-testing/API-TestData/728300_Organization.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Whitelisted\Pra_katalon_webUI0326\FEIAutomation\External_TestData\API\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Whitelisted\Palywright_0409\katalon-to-playwright\testExecution\api-e2e-testing\API-TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{495CCD07-D670-414E-919E-EE8E4CFFDC96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43A02EF9-7D4B-4589-AC2A-8E590A293A22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="860" firstSheet="5" activeTab="9" xr2:uid="{FB437BD9-4435-431A-967E-D926BB2B2714}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="860" xr2:uid="{FB437BD9-4435-431A-967E-D926BB2B2714}"/>
   </bookViews>
   <sheets>
     <sheet name="728300_001_TC001" sheetId="17" r:id="rId1"/>

</xml_diff>